<commit_message>
Fix: Sensor Category/Class/Mode/Technique are set to null for 'None Listed' sensors
</commit_message>
<xml_diff>
--- a/ceos_reformatted_to_smu.xlsx
+++ b/ceos_reformatted_to_smu.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12597" uniqueCount="1492">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12437" uniqueCount="1492">
   <si>
     <t>SatelliteName</t>
   </si>
@@ -5160,18 +5160,6 @@
       <c r="H2" t="s">
         <v>667</v>
       </c>
-      <c r="I2" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J2" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K2" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L2" t="s">
-        <v>809</v>
-      </c>
       <c r="Y2" t="s">
         <v>1159</v>
       </c>
@@ -5494,18 +5482,6 @@
       <c r="H10" t="s">
         <v>667</v>
       </c>
-      <c r="I10" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J10" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K10" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L10" t="s">
-        <v>809</v>
-      </c>
       <c r="Y10" t="s">
         <v>1159</v>
       </c>
@@ -6437,18 +6413,6 @@
       <c r="H30" t="s">
         <v>667</v>
       </c>
-      <c r="I30" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J30" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K30" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L30" t="s">
-        <v>809</v>
-      </c>
       <c r="Y30" t="s">
         <v>1159</v>
       </c>
@@ -11148,18 +11112,6 @@
       <c r="H128" t="s">
         <v>667</v>
       </c>
-      <c r="I128" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J128" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K128" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L128" t="s">
-        <v>809</v>
-      </c>
       <c r="Y128" t="s">
         <v>1159</v>
       </c>
@@ -17976,18 +17928,6 @@
       <c r="H278" t="s">
         <v>667</v>
       </c>
-      <c r="I278" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J278" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K278" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L278" t="s">
-        <v>809</v>
-      </c>
       <c r="O278">
         <v>500</v>
       </c>
@@ -20266,18 +20206,6 @@
       <c r="H325" t="s">
         <v>667</v>
       </c>
-      <c r="I325" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J325" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K325" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L325" t="s">
-        <v>809</v>
-      </c>
       <c r="O325">
         <v>540</v>
       </c>
@@ -20298,18 +20226,6 @@
       <c r="H326" t="s">
         <v>667</v>
       </c>
-      <c r="I326" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J326" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K326" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L326" t="s">
-        <v>809</v>
-      </c>
       <c r="Y326" t="s">
         <v>1159</v>
       </c>
@@ -22478,18 +22394,6 @@
       <c r="H378" t="s">
         <v>667</v>
       </c>
-      <c r="I378" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J378" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K378" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L378" t="s">
-        <v>809</v>
-      </c>
       <c r="O378">
         <v>525</v>
       </c>
@@ -26294,18 +26198,6 @@
       <c r="H459" t="s">
         <v>667</v>
       </c>
-      <c r="I459" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J459" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K459" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L459" t="s">
-        <v>809</v>
-      </c>
       <c r="O459">
         <v>525</v>
       </c>
@@ -27458,18 +27350,6 @@
       <c r="H489" t="s">
         <v>667</v>
       </c>
-      <c r="I489" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J489" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K489" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L489" t="s">
-        <v>809</v>
-      </c>
       <c r="O489">
         <v>35786</v>
       </c>
@@ -27490,18 +27370,6 @@
       <c r="H490" t="s">
         <v>667</v>
       </c>
-      <c r="I490" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J490" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K490" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L490" t="s">
-        <v>809</v>
-      </c>
       <c r="O490">
         <v>613</v>
       </c>
@@ -27522,18 +27390,6 @@
       <c r="H491" t="s">
         <v>667</v>
       </c>
-      <c r="I491" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J491" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K491" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L491" t="s">
-        <v>809</v>
-      </c>
       <c r="O491">
         <v>412</v>
       </c>
@@ -27686,18 +27542,6 @@
       <c r="H495" t="s">
         <v>667</v>
       </c>
-      <c r="I495" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J495" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K495" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L495" t="s">
-        <v>809</v>
-      </c>
       <c r="O495">
         <v>488</v>
       </c>
@@ -27853,18 +27697,6 @@
       <c r="H499" t="s">
         <v>667</v>
       </c>
-      <c r="I499" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J499" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K499" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L499" t="s">
-        <v>809</v>
-      </c>
       <c r="O499">
         <v>475</v>
       </c>
@@ -27885,18 +27717,6 @@
       <c r="H500" t="s">
         <v>667</v>
       </c>
-      <c r="I500" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J500" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K500" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L500" t="s">
-        <v>809</v>
-      </c>
       <c r="O500">
         <v>650</v>
       </c>
@@ -30793,18 +30613,6 @@
       <c r="H571" t="s">
         <v>667</v>
       </c>
-      <c r="I571" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J571" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K571" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L571" t="s">
-        <v>809</v>
-      </c>
       <c r="Y571" t="s">
         <v>1159</v>
       </c>
@@ -31258,18 +31066,6 @@
       <c r="H580" t="s">
         <v>667</v>
       </c>
-      <c r="I580" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J580" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K580" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L580" t="s">
-        <v>809</v>
-      </c>
       <c r="O580">
         <v>500</v>
       </c>
@@ -31290,18 +31086,6 @@
       <c r="H581" t="s">
         <v>667</v>
       </c>
-      <c r="I581" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J581" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K581" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L581" t="s">
-        <v>809</v>
-      </c>
       <c r="O581">
         <v>506</v>
       </c>
@@ -31322,18 +31106,6 @@
       <c r="H582" t="s">
         <v>667</v>
       </c>
-      <c r="I582" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J582" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K582" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L582" t="s">
-        <v>809</v>
-      </c>
       <c r="Y582" t="s">
         <v>1159</v>
       </c>
@@ -32110,18 +31882,6 @@
       <c r="H601" t="s">
         <v>667</v>
       </c>
-      <c r="I601" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J601" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K601" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L601" t="s">
-        <v>809</v>
-      </c>
       <c r="O601">
         <v>640</v>
       </c>
@@ -32189,18 +31949,6 @@
       <c r="H603" t="s">
         <v>667</v>
       </c>
-      <c r="I603" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J603" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K603" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L603" t="s">
-        <v>809</v>
-      </c>
       <c r="O603">
         <v>510</v>
       </c>
@@ -38339,18 +38087,6 @@
       <c r="H741" t="s">
         <v>667</v>
       </c>
-      <c r="I741" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J741" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K741" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L741" t="s">
-        <v>809</v>
-      </c>
       <c r="Y741" t="s">
         <v>1159</v>
       </c>
@@ -41695,18 +41431,6 @@
       <c r="H811" t="s">
         <v>667</v>
       </c>
-      <c r="I811" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J811" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K811" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L811" t="s">
-        <v>809</v>
-      </c>
       <c r="Y811" t="s">
         <v>1159</v>
       </c>
@@ -42190,18 +41914,6 @@
       <c r="H823" t="s">
         <v>667</v>
       </c>
-      <c r="I823" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J823" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K823" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L823" t="s">
-        <v>809</v>
-      </c>
       <c r="O823">
         <v>550</v>
       </c>
@@ -44104,18 +43816,6 @@
       <c r="H865" t="s">
         <v>667</v>
       </c>
-      <c r="I865" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J865" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K865" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L865" t="s">
-        <v>809</v>
-      </c>
       <c r="O865">
         <v>550</v>
       </c>
@@ -44436,18 +44136,6 @@
       <c r="H872" t="s">
         <v>667</v>
       </c>
-      <c r="I872" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J872" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K872" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L872" t="s">
-        <v>809</v>
-      </c>
       <c r="Y872" t="s">
         <v>1159</v>
       </c>
@@ -44465,18 +44153,6 @@
       <c r="H873" t="s">
         <v>667</v>
       </c>
-      <c r="I873" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J873" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K873" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L873" t="s">
-        <v>809</v>
-      </c>
       <c r="Y873" t="s">
         <v>1159</v>
       </c>
@@ -45182,18 +44858,6 @@
       <c r="H888" t="s">
         <v>667</v>
       </c>
-      <c r="I888" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J888" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K888" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L888" t="s">
-        <v>809</v>
-      </c>
       <c r="Y888" t="s">
         <v>1159</v>
       </c>
@@ -49540,18 +49204,6 @@
       <c r="H976" t="s">
         <v>667</v>
       </c>
-      <c r="I976" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J976" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K976" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L976" t="s">
-        <v>809</v>
-      </c>
       <c r="Y976" t="s">
         <v>1159</v>
       </c>
@@ -54451,18 +54103,6 @@
       <c r="H1081" t="s">
         <v>667</v>
       </c>
-      <c r="I1081" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J1081" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K1081" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L1081" t="s">
-        <v>809</v>
-      </c>
       <c r="Y1081" t="s">
         <v>1159</v>
       </c>
@@ -54480,18 +54120,6 @@
       <c r="H1082" t="s">
         <v>667</v>
       </c>
-      <c r="I1082" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J1082" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K1082" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L1082" t="s">
-        <v>809</v>
-      </c>
       <c r="Y1082" t="s">
         <v>1159</v>
       </c>
@@ -56359,18 +55987,6 @@
       <c r="H1126" t="s">
         <v>667</v>
       </c>
-      <c r="I1126" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J1126" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K1126" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L1126" t="s">
-        <v>809</v>
-      </c>
       <c r="Y1126" t="s">
         <v>1159</v>
       </c>
@@ -56494,18 +56110,6 @@
       <c r="H1129" t="s">
         <v>667</v>
       </c>
-      <c r="I1129" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J1129" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K1129" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L1129" t="s">
-        <v>809</v>
-      </c>
       <c r="Y1129" t="s">
         <v>1159</v>
       </c>
@@ -56523,18 +56127,6 @@
       <c r="H1130" t="s">
         <v>667</v>
       </c>
-      <c r="I1130" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J1130" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K1130" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L1130" t="s">
-        <v>809</v>
-      </c>
       <c r="Y1130" t="s">
         <v>1159</v>
       </c>
@@ -56939,18 +56531,6 @@
       <c r="H1140" t="s">
         <v>667</v>
       </c>
-      <c r="I1140" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J1140" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K1140" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L1140" t="s">
-        <v>809</v>
-      </c>
       <c r="Y1140" t="s">
         <v>1159</v>
       </c>
@@ -57080,18 +56660,6 @@
       <c r="H1143" t="s">
         <v>667</v>
       </c>
-      <c r="I1143" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J1143" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K1143" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L1143" t="s">
-        <v>809</v>
-      </c>
       <c r="O1143">
         <v>510</v>
       </c>
@@ -57112,18 +56680,6 @@
       <c r="H1144" t="s">
         <v>667</v>
       </c>
-      <c r="I1144" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J1144" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K1144" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L1144" t="s">
-        <v>809</v>
-      </c>
       <c r="O1144">
         <v>780</v>
       </c>
@@ -57208,18 +56764,6 @@
       <c r="H1147" t="s">
         <v>667</v>
       </c>
-      <c r="I1147" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J1147" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K1147" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L1147" t="s">
-        <v>809</v>
-      </c>
       <c r="O1147">
         <v>800</v>
       </c>
@@ -57240,18 +56784,6 @@
       <c r="H1148" t="s">
         <v>667</v>
       </c>
-      <c r="I1148" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J1148" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K1148" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L1148" t="s">
-        <v>809</v>
-      </c>
       <c r="O1148">
         <v>870</v>
       </c>
@@ -57271,18 +56803,6 @@
       </c>
       <c r="H1149" t="s">
         <v>667</v>
-      </c>
-      <c r="I1149" t="s">
-        <v>1086</v>
-      </c>
-      <c r="J1149" t="s">
-        <v>1088</v>
-      </c>
-      <c r="K1149" t="s">
-        <v>1092</v>
-      </c>
-      <c r="L1149" t="s">
-        <v>809</v>
       </c>
       <c r="Y1149" t="s">
         <v>1159</v>

</xml_diff>